<commit_message>
feat: teste das APIs, melhorar calendario de escalas, ajustar estilos
</commit_message>
<xml_diff>
--- a/api/data/examples/escalas.xlsx
+++ b/api/data/examples/escalas.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10322"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10517"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bibianadibellacostabatista/Documents/Thais/Igen/intranet-pasta/tabelas/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bibianadibellacostabatista/Documents/Thais/Igen/intranet-pasta/projeto-intranet/api/data/examples/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{09000812-5E9D-C245-A7B6-BFC11423A9BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6DCBA5A7-5349-1546-973C-D017ED772623}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="280" yWindow="500" windowWidth="28240" windowHeight="16840" xr2:uid="{FB51C58E-5A24-F542-86D8-C77202F3C061}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="187" uniqueCount="52">
   <si>
     <t>Data</t>
   </si>
@@ -53,17 +53,152 @@
     <t>JULIA, KAMILA</t>
   </si>
   <si>
-    <t>CAMILLA C, DANIELLE, LUIZA, THAIS C</t>
-  </si>
-  <si>
     <t>GUILHERME</t>
+  </si>
+  <si>
+    <t>JOANA, SAMANTHA noturno</t>
+  </si>
+  <si>
+    <t>JOANA, SAMANTHA</t>
+  </si>
+  <si>
+    <t>JOANA, JULIANA, NICOLLY, ADRIANA, CLEIDE, ANDREA, GLAUCIA</t>
+  </si>
+  <si>
+    <t>JULIA, CAMILA B, KARINE</t>
+  </si>
+  <si>
+    <t>KAMILA, THAIS, GISELE D., SANDRA, EDNA, VALENTINA, PEDRO, LUIZA B., NATALIA</t>
+  </si>
+  <si>
+    <t>PALOMA, SAMANTHA, VANDRESSA</t>
+  </si>
+  <si>
+    <t>JOANA, SAMANTHA, CAMILA B, ADRIANA, ANA PAULA, EDER, LORENA, ELISA, REBECA</t>
+  </si>
+  <si>
+    <t>JULIA, JULIANA, KARINE</t>
+  </si>
+  <si>
+    <t>KAMILA, PALOMA, GISELE D, DEBORA, ALAN, FERNANDA, LARISSA</t>
+  </si>
+  <si>
+    <t>THAIS, VANDRESSA, NICOLLY</t>
+  </si>
+  <si>
+    <t>SAMANTHA, MARIA</t>
+  </si>
+  <si>
+    <t>CAMILLA C., LUIZA, TAIMIRIS, DANIELLE, THAIS C</t>
+  </si>
+  <si>
+    <t>ANA, YURI</t>
+  </si>
+  <si>
+    <t>CAMILLA C., DANIELLE, TAMIRIS, LUIZA, THAIS C</t>
+  </si>
+  <si>
+    <t>CAMILLA C., DANIELLE, LUIZA, THAIS C</t>
+  </si>
+  <si>
+    <t>ANA, YURI, MARIA</t>
+  </si>
+  <si>
+    <t>CAMILLA C., TAMIRIS, DANIELLE, THAIS C</t>
+  </si>
+  <si>
+    <t>YURI, MARIA</t>
+  </si>
+  <si>
+    <t>CAMILLA C., LUIZA, TAMIRIS, THAIS C</t>
+  </si>
+  <si>
+    <t>LUIZA, TAMIRIS, DANIELLE</t>
+  </si>
+  <si>
+    <t>ANA, MARIA</t>
+  </si>
+  <si>
+    <t>CAMILLA C., LUIZA, TAMIRIS, DANIELLE, THAIS C</t>
+  </si>
+  <si>
+    <t>YURI, MARIA, MARINA</t>
+  </si>
+  <si>
+    <t>ANA, YURI, MARIA, MARINA</t>
+  </si>
+  <si>
+    <t>LUIZA, TAMIRIS, DANIELLE, THAIS C</t>
+  </si>
+  <si>
+    <t>CAMILLA C., LUIZA, DANIELLE</t>
+  </si>
+  <si>
+    <t>ANA, MARIA, MARINA</t>
+  </si>
+  <si>
+    <t>DANILO</t>
+  </si>
+  <si>
+    <t>JULIA, KAMILA, PALOMA, Sandra, Gláucia (banco horas)</t>
+  </si>
+  <si>
+    <t>JULIANA, VANDRESSA, KARINE</t>
+  </si>
+  <si>
+    <t>THAIS, SAMANTHA, JOANA (plantão noturno), Adriana, Andrea, Luiza B.</t>
+  </si>
+  <si>
+    <t>CAMILA B, JULIA</t>
+  </si>
+  <si>
+    <t>KAMILA, VANDRESSA, Adriana, Cleide, Edna, Valentina, Elisa</t>
+  </si>
+  <si>
+    <t>PALOMA, NICOLLY, JOANA (plantão noturno)</t>
+  </si>
+  <si>
+    <t>CAMILA B, SAMANTHA, Gisele D., Débora, Éder, Pedro, Gláucia, Isaú, Rebeca</t>
+  </si>
+  <si>
+    <t>JOANA (plantão noturno), SAMANTHA</t>
+  </si>
+  <si>
+    <t>KAMILA, NICOLLY, Ana Paula, Gisele D., Alan, Fernanda, Lorena, Larissa, Natália</t>
+  </si>
+  <si>
+    <t>JOANA, THAIS, SAMANTHA</t>
+  </si>
+  <si>
+    <t>TAMIRIS, LUIZA</t>
+  </si>
+  <si>
+    <t>JOANA, MARIA, MARINA</t>
+  </si>
+  <si>
+    <t>CAMILLA C., TAMIRIS, THAIS C</t>
+  </si>
+  <si>
+    <t>CAMILLA C., TAMIRIS, LUIZA, THAIS C</t>
+  </si>
+  <si>
+    <t>CAMILLA C., LUIZA</t>
+  </si>
+  <si>
+    <t>ANA, JOANA, MARINA</t>
+  </si>
+  <si>
+    <t>TAMIRIS, LUIZA, THAIS C</t>
+  </si>
+  <si>
+    <t>CAMILLA C., LUIZA Folga, TAMIRIS, DANIELLE, THAIS C</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -77,13 +212,26 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="3" tint="0.89999084444715716"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -98,10 +246,19 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -436,16 +593,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A72E487D-1DAB-C44D-B5FE-396A53849B39}">
-  <dimension ref="A1:D6"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:D62"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="30" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="33.6640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.1640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.33203125" style="5" customWidth="1"/>
+    <col min="2" max="2" width="69.33203125" style="4" customWidth="1"/>
+    <col min="3" max="3" width="56" style="4" customWidth="1"/>
+    <col min="4" max="4" width="11.1640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="5" max="16384" width="10.83203125" style="4"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
@@ -460,41 +619,857 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A2" s="2">
-        <v>46082</v>
+        <v>46143</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>5</v>
+        <v>18</v>
       </c>
       <c r="D2" s="1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A3" s="2">
+        <v>46144</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A4" s="2">
+        <v>46145</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A5" s="2">
+        <v>46146</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A6" s="2">
+        <v>46147</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A7" s="2">
+        <v>46148</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A8" s="2">
+        <v>46149</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A9" s="2">
+        <v>46150</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A10" s="2">
+        <v>46151</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A11" s="2">
+        <v>46152</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A12" s="2">
+        <v>46153</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A13" s="2">
+        <v>46154</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A14" s="2">
+        <v>46155</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A15" s="2">
+        <v>46156</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A16" s="2">
+        <v>46157</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A17" s="2">
+        <v>46158</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A18" s="2">
+        <v>46159</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A19" s="2">
+        <v>46160</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A20" s="2">
+        <v>46161</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="D20" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A21" s="2">
+        <v>46162</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="D21" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A22" s="2">
+        <v>46163</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="D22" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A23" s="2">
+        <v>46164</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="D23" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A24" s="2">
+        <v>46165</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D24" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A25" s="2">
+        <v>46166</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="D25" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A26" s="2">
+        <v>46167</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="C26" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="D26" s="1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A27" s="2">
+        <v>46168</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C27" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="D27" s="1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A28" s="2">
+        <v>46169</v>
+      </c>
+      <c r="B28" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C28" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="D28" s="1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A29" s="2">
+        <v>46170</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C29" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="D29" s="1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A30" s="2">
+        <v>46171</v>
+      </c>
+      <c r="B30" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C30" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="D30" s="1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A31" s="2">
+        <v>46172</v>
+      </c>
+      <c r="B31" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="C31" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="D31" s="1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A32" s="2">
+        <v>46173</v>
+      </c>
+      <c r="B32" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="C32" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D32" s="1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A33" s="2">
+        <v>46174</v>
+      </c>
+      <c r="B33" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C33" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="D33" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A34" s="2">
+        <v>46175</v>
+      </c>
+      <c r="B34" s="4" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A3" s="2"/>
-      <c r="B3" s="1"/>
-      <c r="C3" s="1"/>
-      <c r="D3" s="1"/>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A4" s="2"/>
-      <c r="B4" s="1"/>
-      <c r="C4" s="1"/>
-      <c r="D4" s="1"/>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A5" s="2"/>
-      <c r="B5" s="1"/>
-      <c r="C5" s="1"/>
-      <c r="D5" s="1"/>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A6" s="2"/>
-      <c r="B6" s="1"/>
-      <c r="C6" s="1"/>
-      <c r="D6" s="1"/>
+      <c r="C34" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="D34" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A35" s="2">
+        <v>46176</v>
+      </c>
+      <c r="B35" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C35" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="D35" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A36" s="2">
+        <v>46177</v>
+      </c>
+      <c r="B36" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C36" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="D36" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A37" s="2">
+        <v>46178</v>
+      </c>
+      <c r="B37" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C37" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D37" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A38" s="3">
+        <v>46179</v>
+      </c>
+      <c r="B38" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C38" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="D38" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A39" s="3">
+        <v>46180</v>
+      </c>
+      <c r="B39" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C39" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="D39" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A40" s="2">
+        <v>46181</v>
+      </c>
+      <c r="B40" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C40" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="D40" s="1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A41" s="2">
+        <v>46182</v>
+      </c>
+      <c r="B41" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C41" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="D41" s="1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A42" s="2">
+        <v>46183</v>
+      </c>
+      <c r="B42" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C42" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="D42" s="1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A43" s="2">
+        <v>46184</v>
+      </c>
+      <c r="B43" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C43" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="D43" s="1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A44" s="2">
+        <v>46185</v>
+      </c>
+      <c r="B44" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C44" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="D44" s="1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A45" s="3">
+        <v>46186</v>
+      </c>
+      <c r="B45" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C45" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="D45" s="1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A46" s="3">
+        <v>46187</v>
+      </c>
+      <c r="B46" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C46" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="D46" s="1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A47" s="2">
+        <v>46188</v>
+      </c>
+      <c r="B47" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C47" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="D47" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A48" s="2">
+        <v>46189</v>
+      </c>
+      <c r="B48" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C48" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="D48" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A49" s="2">
+        <v>46190</v>
+      </c>
+      <c r="B49" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C49" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="D49" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A50" s="2">
+        <v>46191</v>
+      </c>
+      <c r="B50" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C50" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="D50" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A51" s="2">
+        <v>46192</v>
+      </c>
+      <c r="B51" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C51" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="D51" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A52" s="3">
+        <v>46193</v>
+      </c>
+      <c r="B52" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="C52" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="D52" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A53" s="3">
+        <v>46194</v>
+      </c>
+      <c r="B53" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C53" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="D53" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A54" s="2">
+        <v>46195</v>
+      </c>
+      <c r="B54" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C54" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="D54" s="1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A55" s="2">
+        <v>46196</v>
+      </c>
+      <c r="B55" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C55" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="D55" s="1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A56" s="2">
+        <v>46197</v>
+      </c>
+      <c r="B56" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C56" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="D56" s="1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A57" s="2">
+        <v>46198</v>
+      </c>
+      <c r="B57" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C57" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="D57" s="1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A58" s="2">
+        <v>46199</v>
+      </c>
+      <c r="B58" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C58" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="D58" s="1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A59" s="3">
+        <v>46200</v>
+      </c>
+      <c r="B59" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C59" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="D59" s="1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A60" s="3">
+        <v>46201</v>
+      </c>
+      <c r="B60" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="C60" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="D60" s="1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A61" s="2">
+        <v>46202</v>
+      </c>
+      <c r="B61" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C61" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="D61" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A62" s="2">
+        <v>46203</v>
+      </c>
+      <c r="B62" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C62" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="D62" s="1" t="s">
+        <v>5</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>

</xml_diff>

<commit_message>
feat: atualiza planilhas de escalas, ferias e folgas
</commit_message>
<xml_diff>
--- a/api/data/examples/escalas.xlsx
+++ b/api/data/examples/escalas.xlsx
@@ -1,20 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10517"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10525"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bibianadibellacostabatista/Documents/Thais/Igen/intranet-pasta/projeto-intranet/api/data/examples/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6DCBA5A7-5349-1546-973C-D017ED772623}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF8DF9E0-C0C1-1A49-A90A-0E72B030A709}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="280" yWindow="500" windowWidth="28240" windowHeight="16840" xr2:uid="{FB51C58E-5A24-F542-86D8-C77202F3C061}"/>
+    <workbookView xWindow="220" yWindow="1700" windowWidth="28240" windowHeight="16840" xr2:uid="{FB51C58E-5A24-F542-86D8-C77202F3C061}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Planilha1!$A$1:$D$93</definedName>
+  </definedNames>
   <calcPr calcId="181029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -36,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="187" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="280" uniqueCount="75">
   <si>
     <t>Data</t>
   </si>
@@ -50,148 +53,217 @@
     <t>TI (Nomes)</t>
   </si>
   <si>
-    <t>JULIA, KAMILA</t>
-  </si>
-  <si>
-    <t>GUILHERME</t>
-  </si>
-  <si>
-    <t>JOANA, SAMANTHA noturno</t>
-  </si>
-  <si>
-    <t>JOANA, SAMANTHA</t>
-  </si>
-  <si>
-    <t>JOANA, JULIANA, NICOLLY, ADRIANA, CLEIDE, ANDREA, GLAUCIA</t>
-  </si>
-  <si>
-    <t>JULIA, CAMILA B, KARINE</t>
-  </si>
-  <si>
-    <t>KAMILA, THAIS, GISELE D., SANDRA, EDNA, VALENTINA, PEDRO, LUIZA B., NATALIA</t>
-  </si>
-  <si>
-    <t>PALOMA, SAMANTHA, VANDRESSA</t>
-  </si>
-  <si>
-    <t>JOANA, SAMANTHA, CAMILA B, ADRIANA, ANA PAULA, EDER, LORENA, ELISA, REBECA</t>
-  </si>
-  <si>
-    <t>JULIA, JULIANA, KARINE</t>
-  </si>
-  <si>
-    <t>KAMILA, PALOMA, GISELE D, DEBORA, ALAN, FERNANDA, LARISSA</t>
-  </si>
-  <si>
-    <t>THAIS, VANDRESSA, NICOLLY</t>
-  </si>
-  <si>
-    <t>SAMANTHA, MARIA</t>
-  </si>
-  <si>
-    <t>CAMILLA C., LUIZA, TAIMIRIS, DANIELLE, THAIS C</t>
-  </si>
-  <si>
-    <t>ANA, YURI</t>
-  </si>
-  <si>
-    <t>CAMILLA C., DANIELLE, TAMIRIS, LUIZA, THAIS C</t>
-  </si>
-  <si>
-    <t>CAMILLA C., DANIELLE, LUIZA, THAIS C</t>
-  </si>
-  <si>
-    <t>ANA, YURI, MARIA</t>
-  </si>
-  <si>
-    <t>CAMILLA C., TAMIRIS, DANIELLE, THAIS C</t>
-  </si>
-  <si>
-    <t>YURI, MARIA</t>
-  </si>
-  <si>
-    <t>CAMILLA C., LUIZA, TAMIRIS, THAIS C</t>
-  </si>
-  <si>
-    <t>LUIZA, TAMIRIS, DANIELLE</t>
-  </si>
-  <si>
-    <t>ANA, MARIA</t>
-  </si>
-  <si>
-    <t>CAMILLA C., LUIZA, TAMIRIS, DANIELLE, THAIS C</t>
-  </si>
-  <si>
-    <t>YURI, MARIA, MARINA</t>
-  </si>
-  <si>
-    <t>ANA, YURI, MARIA, MARINA</t>
-  </si>
-  <si>
-    <t>LUIZA, TAMIRIS, DANIELLE, THAIS C</t>
-  </si>
-  <si>
-    <t>CAMILLA C., LUIZA, DANIELLE</t>
-  </si>
-  <si>
-    <t>ANA, MARIA, MARINA</t>
-  </si>
-  <si>
-    <t>DANILO</t>
-  </si>
-  <si>
-    <t>JULIA, KAMILA, PALOMA, Sandra, Gláucia (banco horas)</t>
-  </si>
-  <si>
-    <t>JULIANA, VANDRESSA, KARINE</t>
-  </si>
-  <si>
-    <t>THAIS, SAMANTHA, JOANA (plantão noturno), Adriana, Andrea, Luiza B.</t>
-  </si>
-  <si>
-    <t>CAMILA B, JULIA</t>
-  </si>
-  <si>
-    <t>KAMILA, VANDRESSA, Adriana, Cleide, Edna, Valentina, Elisa</t>
-  </si>
-  <si>
-    <t>PALOMA, NICOLLY, JOANA (plantão noturno)</t>
-  </si>
-  <si>
-    <t>CAMILA B, SAMANTHA, Gisele D., Débora, Éder, Pedro, Gláucia, Isaú, Rebeca</t>
-  </si>
-  <si>
-    <t>JOANA (plantão noturno), SAMANTHA</t>
-  </si>
-  <si>
-    <t>KAMILA, NICOLLY, Ana Paula, Gisele D., Alan, Fernanda, Lorena, Larissa, Natália</t>
-  </si>
-  <si>
-    <t>JOANA, THAIS, SAMANTHA</t>
-  </si>
-  <si>
-    <t>TAMIRIS, LUIZA</t>
-  </si>
-  <si>
-    <t>JOANA, MARIA, MARINA</t>
-  </si>
-  <si>
-    <t>CAMILLA C., TAMIRIS, THAIS C</t>
-  </si>
-  <si>
-    <t>CAMILLA C., TAMIRIS, LUIZA, THAIS C</t>
-  </si>
-  <si>
-    <t>CAMILLA C., LUIZA</t>
-  </si>
-  <si>
-    <t>ANA, JOANA, MARINA</t>
-  </si>
-  <si>
-    <t>TAMIRIS, LUIZA, THAIS C</t>
-  </si>
-  <si>
-    <t>CAMILLA C., LUIZA Folga, TAMIRIS, DANIELLE, THAIS C</t>
+    <t>Joana, Samantha</t>
+  </si>
+  <si>
+    <t>Ana, Yuri</t>
+  </si>
+  <si>
+    <t>Julia, Kamila, Paloma, Sandra, Gláucia (banco Horas)</t>
+  </si>
+  <si>
+    <t>Tamiris, Luiza</t>
+  </si>
+  <si>
+    <t>Juliana, Vandressa, Karine</t>
+  </si>
+  <si>
+    <t>Ana, Maria, Marina</t>
+  </si>
+  <si>
+    <t>Julia, Kamila</t>
+  </si>
+  <si>
+    <t>Camilla C., Luiza, Tamiris, Thais C</t>
+  </si>
+  <si>
+    <t>Camilla C., Luiza, Tamiris, Danielle, Thais C</t>
+  </si>
+  <si>
+    <t>Thais, Samantha, Joana (plantão Noturno), Adriana, Andrea, Luiza B.</t>
+  </si>
+  <si>
+    <t>Joana, Maria, Marina</t>
+  </si>
+  <si>
+    <t>Camila B, Julia</t>
+  </si>
+  <si>
+    <t>Camilla C., Tamiris, Thais C</t>
+  </si>
+  <si>
+    <t>Camilla C., Tamiris, Luiza, Thais C</t>
+  </si>
+  <si>
+    <t>Kamila, Vandressa, Adriana, Cleide, Edna, Valentina, Elisa</t>
+  </si>
+  <si>
+    <t>Camilla C., Luiza</t>
+  </si>
+  <si>
+    <t>Paloma, Nicolly, Joana (plantão Noturno)</t>
+  </si>
+  <si>
+    <t>Ana, Joana, Marina</t>
+  </si>
+  <si>
+    <t>Camila B, Samantha, Gisele D., Débora, Éder, Pedro, Gláucia, Isaú, Rebeca</t>
+  </si>
+  <si>
+    <t>Ana, Maria</t>
+  </si>
+  <si>
+    <t>Julia, Juliana, Karine</t>
+  </si>
+  <si>
+    <t>Joana (plantão Noturno), Samantha</t>
+  </si>
+  <si>
+    <t>Kamila, Nicolly, Ana Paula, Gisele D., Alan, Fernanda, Lorena, Larissa, Natália</t>
+  </si>
+  <si>
+    <t>Tamiris, Luiza, Thais C</t>
+  </si>
+  <si>
+    <t>Joana, Thais, Samantha</t>
+  </si>
+  <si>
+    <t>Julia</t>
+  </si>
+  <si>
+    <t>Camilla C., Luiza, Taimiris, Danielle, Thais C</t>
+  </si>
+  <si>
+    <t>Samantha, Maria</t>
+  </si>
+  <si>
+    <t>Camilla C., Danielle, Tamiris, Luiza, Thais C</t>
+  </si>
+  <si>
+    <t>Joana, Juliana, Nicolly, Adriana, Cleide, Andrea, Gláucia</t>
+  </si>
+  <si>
+    <t>Julia, Camila B, Karine</t>
+  </si>
+  <si>
+    <t>Camilla C., Danielle, Luiza, Thais C</t>
+  </si>
+  <si>
+    <t>Ana, Yuri, Maria</t>
+  </si>
+  <si>
+    <t>Camilla C., Tamiris, Danielle, Thais C</t>
+  </si>
+  <si>
+    <t>Yuri, Maria</t>
+  </si>
+  <si>
+    <t>Thais, Vandressa, Gisele D., Sandra, Edna, Valentina, Pedro, Luiza B., Natália</t>
+  </si>
+  <si>
+    <t>Luiza, Tamiris, Danielle</t>
+  </si>
+  <si>
+    <t>Paloma, Samantha</t>
+  </si>
+  <si>
+    <t>Joana, Samantha, Camila B, Adriana, Ana Paula, Éder, Lorena, Elisa, Rebeca</t>
+  </si>
+  <si>
+    <t>Camilla C., Luiza, Danielle</t>
+  </si>
+  <si>
+    <t>Ana, Yuri, Maria, Marina</t>
+  </si>
+  <si>
+    <t>Yuri, Maria, Marina</t>
+  </si>
+  <si>
+    <t>Paloma, Nicolly, Gisele D., Débora, Alan, Fernanda, Larissa</t>
+  </si>
+  <si>
+    <t>Thais, Vandressa</t>
+  </si>
+  <si>
+    <t>Luiza, Tamiris, Danielle, Thais C</t>
+  </si>
+  <si>
+    <t>Danilo</t>
+  </si>
+  <si>
+    <t>Guilherme</t>
+  </si>
+  <si>
+    <t>Joana, Samantha faz plantão noturno</t>
+  </si>
+  <si>
+    <t>Guilhermme</t>
+  </si>
+  <si>
+    <t>Camilla C., Luiza, Tamiris, Danielle, Thais C.</t>
+  </si>
+  <si>
+    <t>Joana, Karine, Samantha, Adriana, Gisele D., Eder, Lorena, Fernanda, Elisa, Natalia</t>
+  </si>
+  <si>
+    <t>Camila B., Julia</t>
+  </si>
+  <si>
+    <t>Camilla C., Tamiris, Danielle, Thais C.</t>
+  </si>
+  <si>
+    <t>Joana</t>
+  </si>
+  <si>
+    <t>Julia, Thais (Extra)</t>
+  </si>
+  <si>
+    <t>Camilla C., Luiza, Tamiris, Thais C.</t>
+  </si>
+  <si>
+    <t>Yuri, Maria, Ana, Marina</t>
+  </si>
+  <si>
+    <t>Vandressa, Thais, Ana Paula, Debora (8h), Alan, Isau</t>
+  </si>
+  <si>
+    <t>Joana, Paloma, Samantha</t>
+  </si>
+  <si>
+    <t>Ana, Maria, Yuri, Marina</t>
+  </si>
+  <si>
+    <t>Camilla C., Luiza, Danielle, Thais C.</t>
+  </si>
+  <si>
+    <t>Joana, Nicolly, Gisele D., Sandra, Edna, Valentina, Larissa, Rebeca</t>
+  </si>
+  <si>
+    <t>Maria, Yuri</t>
+  </si>
+  <si>
+    <t>Camila B., Julia, Karine</t>
+  </si>
+  <si>
+    <t>Camilla C., Luiza, Thais C.</t>
+  </si>
+  <si>
+    <t>Paloma, Juliana, Adriana, Cleide, Andrea, Gláucia, Pedro, Luiza B.</t>
+  </si>
+  <si>
+    <t>Luiza, Danielle</t>
+  </si>
+  <si>
+    <t>Samantha</t>
+  </si>
+  <si>
+    <t>Ana, Yuri, Marina</t>
+  </si>
+  <si>
+    <t>Camilla C., Tamiris, Thais C.</t>
+  </si>
+  <si>
+    <t>Camilla C., Danielle, Thais C.</t>
   </si>
 </sst>
 </file>
@@ -593,7 +665,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A72E487D-1DAB-C44D-B5FE-396A53849B39}">
-  <dimension ref="A1:D62"/>
+  <dimension ref="A1:D93"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="14.33203125" style="5" customWidth="1"/>
@@ -622,13 +694,13 @@
         <v>46143</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>18</v>
+        <v>5</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>33</v>
+        <v>49</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.2">
@@ -636,13 +708,13 @@
         <v>46144</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>34</v>
+        <v>6</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>44</v>
+        <v>7</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>33</v>
+        <v>49</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
@@ -650,13 +722,13 @@
         <v>46145</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>35</v>
+        <v>8</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>32</v>
+        <v>9</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>33</v>
+        <v>49</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
@@ -664,13 +736,13 @@
         <v>46146</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>24</v>
+        <v>11</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>5</v>
+        <v>50</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.2">
@@ -678,13 +750,13 @@
         <v>46147</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>32</v>
+        <v>9</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>5</v>
+        <v>50</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.2">
@@ -692,13 +764,13 @@
         <v>46148</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>51</v>
+        <v>37</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>5</v>
+        <v>50</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.2">
@@ -706,13 +778,13 @@
         <v>46149</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>32</v>
+        <v>9</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>5</v>
+        <v>50</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.2">
@@ -720,13 +792,13 @@
         <v>46150</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>5</v>
+        <v>50</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.2">
@@ -734,13 +806,13 @@
         <v>46151</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>36</v>
+        <v>13</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>45</v>
+        <v>14</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>5</v>
+        <v>50</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.2">
@@ -748,13 +820,13 @@
         <v>46152</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>37</v>
+        <v>15</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>46</v>
+        <v>16</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>5</v>
+        <v>50</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.2">
@@ -762,13 +834,13 @@
         <v>46153</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>32</v>
+        <v>9</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>33</v>
+        <v>49</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.2">
@@ -776,13 +848,13 @@
         <v>46154</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>47</v>
+        <v>17</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>33</v>
+        <v>49</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.2">
@@ -790,13 +862,13 @@
         <v>46155</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>32</v>
+        <v>9</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>33</v>
+        <v>49</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.2">
@@ -804,13 +876,13 @@
         <v>46156</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>47</v>
+        <v>17</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>33</v>
+        <v>49</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.2">
@@ -818,13 +890,13 @@
         <v>46157</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>32</v>
+        <v>9</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>33</v>
+        <v>49</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.2">
@@ -832,13 +904,13 @@
         <v>46158</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>38</v>
+        <v>18</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>48</v>
+        <v>19</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>33</v>
+        <v>49</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.2">
@@ -846,13 +918,13 @@
         <v>46159</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>39</v>
+        <v>20</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>49</v>
+        <v>21</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>33</v>
+        <v>49</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.2">
@@ -860,13 +932,13 @@
         <v>46160</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>47</v>
+        <v>17</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>5</v>
+        <v>50</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.2">
@@ -874,13 +946,13 @@
         <v>46161</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>32</v>
+        <v>9</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>5</v>
+        <v>50</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.2">
@@ -888,13 +960,13 @@
         <v>46162</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>47</v>
+        <v>17</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>5</v>
+        <v>50</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.2">
@@ -902,13 +974,13 @@
         <v>46163</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>32</v>
+        <v>9</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>5</v>
+        <v>50</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.2">
@@ -916,13 +988,13 @@
         <v>46164</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>47</v>
+        <v>17</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>5</v>
+        <v>50</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.2">
@@ -930,13 +1002,13 @@
         <v>46165</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>40</v>
+        <v>22</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>5</v>
+        <v>50</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.2">
@@ -944,13 +1016,13 @@
         <v>46166</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>46</v>
+        <v>16</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>5</v>
+        <v>50</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.2">
@@ -958,13 +1030,13 @@
         <v>46167</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>41</v>
+        <v>25</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>45</v>
+        <v>14</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>33</v>
+        <v>49</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.2">
@@ -972,13 +1044,13 @@
         <v>46168</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>47</v>
+        <v>17</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>33</v>
+        <v>49</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.2">
@@ -986,13 +1058,13 @@
         <v>46169</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>32</v>
+        <v>9</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>33</v>
+        <v>49</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.2">
@@ -1000,13 +1072,13 @@
         <v>46170</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>47</v>
+        <v>17</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>33</v>
+        <v>49</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.2">
@@ -1014,13 +1086,13 @@
         <v>46171</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>32</v>
+        <v>9</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>33</v>
+        <v>49</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.2">
@@ -1028,13 +1100,13 @@
         <v>46172</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>42</v>
+        <v>26</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>50</v>
+        <v>27</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>33</v>
+        <v>49</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.2">
@@ -1042,13 +1114,13 @@
         <v>46173</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>43</v>
+        <v>28</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>33</v>
+        <v>49</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.2">
@@ -1056,419 +1128,853 @@
         <v>46174</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="C33" s="4" t="s">
-        <v>17</v>
+        <v>29</v>
+      </c>
+      <c r="C33" s="1" t="s">
+        <v>30</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>5</v>
+        <v>50</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A34" s="2">
         <v>46175</v>
       </c>
-      <c r="B34" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="C34" s="4" t="s">
-        <v>16</v>
+      <c r="B34" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="C34" s="1" t="s">
+        <v>31</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>5</v>
+        <v>50</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A35" s="2">
         <v>46176</v>
       </c>
-      <c r="B35" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="C35" s="4" t="s">
-        <v>17</v>
+      <c r="B35" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C35" s="1" t="s">
+        <v>30</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>5</v>
+        <v>50</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A36" s="2">
         <v>46177</v>
       </c>
-      <c r="B36" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="C36" s="4" t="s">
-        <v>18</v>
+      <c r="B36" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C36" s="1" t="s">
+        <v>5</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>5</v>
+        <v>50</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A37" s="2">
         <v>46178</v>
       </c>
-      <c r="B37" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="C37" s="4" t="s">
-        <v>19</v>
+      <c r="B37" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C37" s="1" t="s">
+        <v>32</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>5</v>
+        <v>50</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A38" s="3">
         <v>46179</v>
       </c>
-      <c r="B38" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="C38" s="4" t="s">
-        <v>18</v>
+      <c r="B38" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C38" s="1" t="s">
+        <v>5</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>5</v>
+        <v>50</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A39" s="3">
         <v>46180</v>
       </c>
-      <c r="B39" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="C39" s="4" t="s">
-        <v>20</v>
+      <c r="B39" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="C39" s="1" t="s">
+        <v>35</v>
       </c>
       <c r="D39" s="1" t="s">
-        <v>5</v>
+        <v>50</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A40" s="2">
         <v>46181</v>
       </c>
-      <c r="B40" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="C40" s="4" t="s">
-        <v>21</v>
+      <c r="B40" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C40" s="1" t="s">
+        <v>36</v>
       </c>
       <c r="D40" s="1" t="s">
-        <v>33</v>
+        <v>49</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A41" s="2">
         <v>46182</v>
       </c>
-      <c r="B41" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="C41" s="4" t="s">
-        <v>22</v>
+      <c r="B41" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C41" s="1" t="s">
+        <v>37</v>
       </c>
       <c r="D41" s="1" t="s">
-        <v>33</v>
+        <v>49</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A42" s="2">
         <v>46183</v>
       </c>
-      <c r="B42" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="C42" s="4" t="s">
-        <v>23</v>
+      <c r="B42" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C42" s="1" t="s">
+        <v>38</v>
       </c>
       <c r="D42" s="1" t="s">
-        <v>33</v>
+        <v>49</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A43" s="2">
         <v>46184</v>
       </c>
-      <c r="B43" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="C43" s="4" t="s">
-        <v>24</v>
+      <c r="B43" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C43" s="1" t="s">
+        <v>11</v>
       </c>
       <c r="D43" s="1" t="s">
-        <v>33</v>
+        <v>49</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A44" s="2">
         <v>46185</v>
       </c>
-      <c r="B44" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="C44" s="4" t="s">
-        <v>23</v>
+      <c r="B44" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C44" s="1" t="s">
+        <v>38</v>
       </c>
       <c r="D44" s="1" t="s">
-        <v>33</v>
+        <v>49</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A45" s="3">
         <v>46186</v>
       </c>
-      <c r="B45" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="C45" s="4" t="s">
-        <v>25</v>
+      <c r="B45" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="C45" s="1" t="s">
+        <v>40</v>
       </c>
       <c r="D45" s="1" t="s">
-        <v>33</v>
+        <v>49</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A46" s="3">
         <v>46187</v>
       </c>
-      <c r="B46" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="C46" s="4" t="s">
-        <v>26</v>
+      <c r="B46" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="C46" s="1" t="s">
+        <v>23</v>
       </c>
       <c r="D46" s="1" t="s">
-        <v>33</v>
+        <v>49</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A47" s="2">
         <v>46188</v>
       </c>
-      <c r="B47" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="C47" s="4" t="s">
-        <v>27</v>
+      <c r="B47" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C47" s="1" t="s">
+        <v>12</v>
       </c>
       <c r="D47" s="1" t="s">
-        <v>5</v>
+        <v>50</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A48" s="2">
         <v>46189</v>
       </c>
-      <c r="B48" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="C48" s="4" t="s">
-        <v>21</v>
+      <c r="B48" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C48" s="1" t="s">
+        <v>36</v>
       </c>
       <c r="D48" s="1" t="s">
-        <v>5</v>
+        <v>50</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A49" s="2">
         <v>46190</v>
       </c>
-      <c r="B49" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="C49" s="4" t="s">
-        <v>27</v>
+      <c r="B49" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C49" s="1" t="s">
+        <v>12</v>
       </c>
       <c r="D49" s="1" t="s">
-        <v>5</v>
+        <v>50</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A50" s="2">
         <v>46191</v>
       </c>
-      <c r="B50" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="C50" s="4" t="s">
-        <v>21</v>
+      <c r="B50" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C50" s="1" t="s">
+        <v>36</v>
       </c>
       <c r="D50" s="1" t="s">
-        <v>5</v>
+        <v>50</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A51" s="2">
         <v>46192</v>
       </c>
-      <c r="B51" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="C51" s="4" t="s">
-        <v>22</v>
+      <c r="B51" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C51" s="1" t="s">
+        <v>37</v>
       </c>
       <c r="D51" s="1" t="s">
-        <v>5</v>
+        <v>50</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A52" s="3">
         <v>46193</v>
       </c>
-      <c r="B52" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="C52" s="4" t="s">
-        <v>18</v>
+      <c r="B52" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="C52" s="1" t="s">
+        <v>5</v>
       </c>
       <c r="D52" s="1" t="s">
-        <v>5</v>
+        <v>50</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A53" s="3">
         <v>46194</v>
       </c>
-      <c r="B53" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="C53" s="4" t="s">
-        <v>31</v>
+      <c r="B53" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C53" s="1" t="s">
+        <v>43</v>
       </c>
       <c r="D53" s="1" t="s">
-        <v>5</v>
+        <v>50</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A54" s="2">
         <v>46195</v>
       </c>
-      <c r="B54" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="C54" s="4" t="s">
-        <v>21</v>
+      <c r="B54" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C54" s="1" t="s">
+        <v>36</v>
       </c>
       <c r="D54" s="1" t="s">
-        <v>33</v>
+        <v>49</v>
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A55" s="2">
         <v>46196</v>
       </c>
-      <c r="B55" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="C55" s="4" t="s">
-        <v>27</v>
+      <c r="B55" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C55" s="1" t="s">
+        <v>12</v>
       </c>
       <c r="D55" s="1" t="s">
-        <v>33</v>
+        <v>49</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A56" s="2">
         <v>46197</v>
       </c>
-      <c r="B56" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="C56" s="4" t="s">
-        <v>29</v>
+      <c r="B56" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C56" s="1" t="s">
+        <v>44</v>
       </c>
       <c r="D56" s="1" t="s">
-        <v>33</v>
+        <v>49</v>
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A57" s="2">
         <v>46198</v>
       </c>
-      <c r="B57" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="C57" s="4" t="s">
-        <v>27</v>
+      <c r="B57" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C57" s="1" t="s">
+        <v>12</v>
       </c>
       <c r="D57" s="1" t="s">
-        <v>33</v>
+        <v>49</v>
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A58" s="2">
         <v>46199</v>
       </c>
-      <c r="B58" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="C58" s="4" t="s">
-        <v>28</v>
+      <c r="B58" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C58" s="1" t="s">
+        <v>45</v>
       </c>
       <c r="D58" s="1" t="s">
-        <v>33</v>
+        <v>49</v>
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A59" s="3">
         <v>46200</v>
       </c>
-      <c r="B59" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="C59" s="4" t="s">
-        <v>24</v>
+      <c r="B59" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C59" s="1" t="s">
+        <v>11</v>
       </c>
       <c r="D59" s="1" t="s">
-        <v>33</v>
+        <v>49</v>
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A60" s="3">
         <v>46201</v>
       </c>
-      <c r="B60" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="C60" s="4" t="s">
-        <v>29</v>
+      <c r="B60" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="C60" s="1" t="s">
+        <v>44</v>
       </c>
       <c r="D60" s="1" t="s">
-        <v>33</v>
+        <v>49</v>
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A61" s="2">
         <v>46202</v>
       </c>
-      <c r="B61" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="C61" s="4" t="s">
-        <v>30</v>
+      <c r="B61" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C61" s="1" t="s">
+        <v>48</v>
       </c>
       <c r="D61" s="1" t="s">
-        <v>5</v>
+        <v>50</v>
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A62" s="2">
         <v>46203</v>
       </c>
-      <c r="B62" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="C62" s="4" t="s">
-        <v>32</v>
+      <c r="B62" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C62" s="1" t="s">
+        <v>9</v>
       </c>
       <c r="D62" s="1" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A63" s="2">
+        <v>46204</v>
+      </c>
+      <c r="B63" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C63" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="D63" s="1" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="64" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A64" s="2">
+        <v>46205</v>
+      </c>
+      <c r="B64" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C64" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="D64" s="1" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="65" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A65" s="2">
+        <v>46206</v>
+      </c>
+      <c r="B65" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C65" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="D65" s="1" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="66" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A66" s="2">
+        <v>46207</v>
+      </c>
+      <c r="B66" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="C66" s="1" t="s">
         <v>5</v>
+      </c>
+      <c r="D66" s="1" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="67" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A67" s="2">
+        <v>46208</v>
+      </c>
+      <c r="B67" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="C67" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="D67" s="1" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="68" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A68" s="2">
+        <v>46209</v>
+      </c>
+      <c r="B68" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="C68" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="D68" s="1" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="69" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A69" s="2">
+        <v>46210</v>
+      </c>
+      <c r="B69" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C69" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="D69" s="1" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="70" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A70" s="2">
+        <v>46211</v>
+      </c>
+      <c r="B70" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C70" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D70" s="1" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="71" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A71" s="2">
+        <v>46212</v>
+      </c>
+      <c r="B71" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="C71" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="D71" s="1" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="72" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A72" s="2">
+        <v>46213</v>
+      </c>
+      <c r="B72" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="C72" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="D72" s="1" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="73" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A73" s="2">
+        <v>46214</v>
+      </c>
+      <c r="B73" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="C73" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="D73" s="1" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="74" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A74" s="2">
+        <v>46215</v>
+      </c>
+      <c r="B74" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="C74" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="D74" s="1" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="75" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A75" s="2">
+        <v>46216</v>
+      </c>
+      <c r="B75" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C75" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="D75" s="1" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="76" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A76" s="2">
+        <v>46217</v>
+      </c>
+      <c r="B76" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C76" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="D76" s="1" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="77" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A77" s="2">
+        <v>46218</v>
+      </c>
+      <c r="B77" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C77" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="D77" s="1" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="78" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A78" s="2">
+        <v>46219</v>
+      </c>
+      <c r="B78" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C78" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="D78" s="1" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="79" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A79" s="2">
+        <v>46220</v>
+      </c>
+      <c r="B79" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C79" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="D79" s="1" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="80" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A80" s="2">
+        <v>46221</v>
+      </c>
+      <c r="B80" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="C80" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="D80" s="1" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="81" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A81" s="2">
+        <v>46222</v>
+      </c>
+      <c r="B81" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="C81" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="D81" s="1" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="82" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A82" s="2">
+        <v>46223</v>
+      </c>
+      <c r="B82" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="C82" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="D82" s="1" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="83" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A83" s="2">
+        <v>46224</v>
+      </c>
+      <c r="B83" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C83" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="D83" s="1" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="84" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A84" s="2">
+        <v>46225</v>
+      </c>
+      <c r="B84" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="C84" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="D84" s="1" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="85" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A85" s="2">
+        <v>46226</v>
+      </c>
+      <c r="B85" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C85" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="D85" s="1" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="86" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A86" s="2">
+        <v>46227</v>
+      </c>
+      <c r="B86" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="C86" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="D86" s="1" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="87" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A87" s="2">
+        <v>46228</v>
+      </c>
+      <c r="B87" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="C87" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="D87" s="1" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="88" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A88" s="2">
+        <v>46229</v>
+      </c>
+      <c r="B88" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="C88" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D88" s="1" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="89" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A89" s="2">
+        <v>46230</v>
+      </c>
+      <c r="B89" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C89" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="D89" s="1" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="90" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A90" s="2">
+        <v>46231</v>
+      </c>
+      <c r="B90" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C90" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="D90" s="1" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="91" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A91" s="2">
+        <v>46232</v>
+      </c>
+      <c r="B91" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C91" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="D91" s="1" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="92" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A92" s="2">
+        <v>46233</v>
+      </c>
+      <c r="B92" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C92" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="D92" s="1" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="93" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A93" s="2">
+        <v>46234</v>
+      </c>
+      <c r="B93" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C93" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="D93" s="1" t="s">
+        <v>50</v>
       </c>
     </row>
   </sheetData>

</xml_diff>